<commit_message>
Update Case_test infinite horizon results
</commit_message>
<xml_diff>
--- a/Case_test/Plot/obj.xlsx
+++ b/Case_test/Plot/obj.xlsx
@@ -559,16 +559,16 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>904.0023927072846</v>
+        <v>904.0012719964893</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>1555.110229136274</v>
+        <v>1555.110924532686</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1555.105715344624</v>
+        <v>1555.105716566128</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1555.105717277688</v>
+        <v>1555.10571656613</v>
       </c>
       <c r="F4" s="3">
         <f>SUM(B4:E4)</f>

</xml_diff>